<commit_message>
take ABO comments 70eb52be67902ad1caa9c12fcdae56d3768bbd91
</commit_message>
<xml_diff>
--- a/nr-update-valueset/ig/CodeSystem-as-cs-intern-id-systems.xlsx
+++ b/nr-update-valueset/ig/CodeSystem-as-cs-intern-id-systems.xlsx
@@ -57,13 +57,13 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-06T14:32:05+00:00</t>
+    <t>2024-03-06T16:49:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
   </si>
   <si>
-    <t>ANS</t>
+    <t>Agence du Numérique en Santé (ANS) - 2-10 Rue d'Oradour-sur-Glane, 75015 Paris</t>
   </si>
   <si>
     <t>Contact</t>

</xml_diff>